<commit_message>
Added ScanController with Scan & Clear request
</commit_message>
<xml_diff>
--- a/spring-app/data/monthly-controls/Controle_Janvier_2026.xlsx
+++ b/spring-app/data/monthly-controls/Controle_Janvier_2026.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="51">
   <si>
     <t>ID Alitracer</t>
   </si>
@@ -147,6 +147,24 @@
   </si>
   <si>
     <t>13/01/2026 14:50</t>
+  </si>
+  <si>
+    <t>15/01/2026 10:57</t>
+  </si>
+  <si>
+    <t>15/01/2026 13:21</t>
+  </si>
+  <si>
+    <t>15/01/2026 13:34</t>
+  </si>
+  <si>
+    <t>15/01/2026 13:39</t>
+  </si>
+  <si>
+    <t>15/01/2026 13:40</t>
+  </si>
+  <si>
+    <t>28/01/2026 08:30</t>
   </si>
 </sst>
 </file>
@@ -301,7 +319,7 @@
         <v>13</v>
       </c>
       <c r="H2" t="s" s="0">
-        <v>14</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3">
@@ -327,7 +345,7 @@
         <v>13</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>14</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4">
@@ -341,7 +359,7 @@
         <v>17</v>
       </c>
       <c r="D4" t="n" s="0">
-        <v>11.0</v>
+        <v>12.0</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>11</v>
@@ -353,7 +371,7 @@
         <v>13</v>
       </c>
       <c r="H4" t="s" s="0">
-        <v>14</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -483,7 +501,7 @@
         <v>13</v>
       </c>
       <c r="H9" t="s" s="0">
-        <v>27</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10">
@@ -535,7 +553,7 @@
         <v>13</v>
       </c>
       <c r="H11" t="s" s="0">
-        <v>27</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12">
@@ -665,7 +683,7 @@
         <v>13</v>
       </c>
       <c r="H16" t="s" s="0">
-        <v>34</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17">

</xml_diff>